<commit_message>
Updated list with Marco's UI
</commit_message>
<xml_diff>
--- a/Documentation/3D Asset List.xlsx
+++ b/Documentation/3D Asset List.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Repos\HotelSimulator\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9376DD28-DF76-433B-9F50-8DAA7BBF9F3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A07E6679-A43C-4626-9D34-0B017178647E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Items" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="98">
   <si>
     <t>Item</t>
   </si>
@@ -312,6 +312,18 @@
   </si>
   <si>
     <t>Sprite</t>
+  </si>
+  <si>
+    <t>Save Button</t>
+  </si>
+  <si>
+    <t>Menu Function Button</t>
+  </si>
+  <si>
+    <t>Menu Logo</t>
+  </si>
+  <si>
+    <t>Menu Box Backround</t>
   </si>
 </sst>
 </file>
@@ -629,8 +641,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="46.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -719,9 +742,131 @@
         <v>18</v>
       </c>
     </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H4" t="s">
+        <v>43</v>
+      </c>
+      <c r="I4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D5" t="s">
+        <v>24</v>
+      </c>
+      <c r="G5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" t="s">
+        <v>43</v>
+      </c>
+      <c r="I5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C6" t="s">
+        <v>85</v>
+      </c>
+      <c r="D6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G6" t="s">
+        <v>33</v>
+      </c>
+      <c r="H6" t="s">
+        <v>43</v>
+      </c>
+      <c r="I6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>97</v>
+      </c>
+      <c r="C7" t="s">
+        <v>85</v>
+      </c>
+      <c r="D7" t="s">
+        <v>24</v>
+      </c>
+      <c r="G7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" t="s">
+        <v>43</v>
+      </c>
+      <c r="I7" t="s">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="6">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{44F922AF-9E72-4DC1-B554-102FF6F149AF}">
+          <x14:formula1>
+            <xm:f>Options!$F$2:$F$23</xm:f>
+          </x14:formula1>
+          <xm:sqref>C2:C29</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{8EBC5C2D-FDEB-4C6C-BC41-E937E1C01990}">
+          <x14:formula1>
+            <xm:f>Options!$E$2:$E$22</xm:f>
+          </x14:formula1>
+          <xm:sqref>D2:D39</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{8E676CD5-7802-47B5-8C36-94D89D7FB0C1}">
+          <x14:formula1>
+            <xm:f>Options!$D$2:$D$29</xm:f>
+          </x14:formula1>
+          <xm:sqref>E2:E30</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F81DFD1A-8721-4001-BEF6-4D5E43611D44}">
+          <x14:formula1>
+            <xm:f>Options!$A$2:$A$24</xm:f>
+          </x14:formula1>
+          <xm:sqref>G2:G22</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{2C5C086D-F887-4964-B7CD-F528E5E67B48}">
+          <x14:formula1>
+            <xm:f>Options!$B$2:$B$28</xm:f>
+          </x14:formula1>
+          <xm:sqref>H2:H19</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{77559DAA-2BEB-4F05-9536-33CDB5C24566}">
+          <x14:formula1>
+            <xm:f>Options!$C$2:$C$22</xm:f>
+          </x14:formula1>
+          <xm:sqref>I2:I20</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Updated documents and made sign epxorts
</commit_message>
<xml_diff>
--- a/Documentation/3D Asset List.xlsx
+++ b/Documentation/3D Asset List.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Repos\HotelSimulator\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A07E6679-A43C-4626-9D34-0B017178647E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA247C4A-2929-4FF2-915B-475CA1AC455D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="109">
   <si>
     <t>Item</t>
   </si>
@@ -324,6 +324,39 @@
   </si>
   <si>
     <t>Menu Box Backround</t>
+  </si>
+  <si>
+    <t>Officer Chair</t>
+  </si>
+  <si>
+    <t>Office Desk</t>
+  </si>
+  <si>
+    <t>Keyboard</t>
+  </si>
+  <si>
+    <t>Mouse (Computer)</t>
+  </si>
+  <si>
+    <t>Monitor</t>
+  </si>
+  <si>
+    <t>Stabler</t>
+  </si>
+  <si>
+    <t>Phone</t>
+  </si>
+  <si>
+    <t>Pen</t>
+  </si>
+  <si>
+    <t>Note Pad</t>
+  </si>
+  <si>
+    <t>Sticky Notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fire Extinguisher </t>
   </si>
 </sst>
 </file>
@@ -641,7 +674,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
@@ -820,6 +853,61 @@
       </c>
       <c r="I7" t="s">
         <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated desk status in 3D Asset List
</commit_message>
<xml_diff>
--- a/Documentation/3D Asset List.xlsx
+++ b/Documentation/3D Asset List.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Repos\HotelSimulator\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA247C4A-2929-4FF2-915B-475CA1AC455D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D84B480-6101-4C04-9BE7-2F205679643D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="111">
   <si>
     <t>Item</t>
   </si>
@@ -357,6 +357,12 @@
   </si>
   <si>
     <t xml:space="preserve">Fire Extinguisher </t>
+  </si>
+  <si>
+    <t>Main desk in reception</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/drive/folders/1zRriSyxyTsEwrirwBndouaXDlCC6xlqv?usp=drive_link</t>
   </si>
 </sst>
 </file>
@@ -864,6 +870,30 @@
       <c r="A9" t="s">
         <v>99</v>
       </c>
+      <c r="B9" t="s">
+        <v>109</v>
+      </c>
+      <c r="C9" t="s">
+        <v>88</v>
+      </c>
+      <c r="D9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9" t="s">
+        <v>57</v>
+      </c>
+      <c r="F9" t="s">
+        <v>110</v>
+      </c>
+      <c r="G9" t="s">
+        <v>34</v>
+      </c>
+      <c r="H9" t="s">
+        <v>43</v>
+      </c>
+      <c r="I9" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">

</xml_diff>